<commit_message>
v2: facturas cruzan por documento_operacion_id (MRCLP: Geneva antepone RC), morosas con tasa×12 y duration 0, monto vs cantidad
- fuentes/facturas.py: el número del nombre del CUBO (FACRCPP59397 / FAC68135) es documento_operacion_id y manda; HOMOL de respaldo
- morosas (vencidas y no pagadas al cierre): yield tasa × 12, duration factura_morosa_duration (0), alerta INFO FACTURA_MOROSA
- FACTURA_MONTO_DISTINTO compara monto_compra con Qty (nominal), no con el MV a precio con devengo
- README y PLAN con el diagnóstico de la corrida real (730 facturas faltantes: 473 MRCLP por nombre, 185 morosas)

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MSSQoFR1coHjRzkTJJ7d3F
</commit_message>
<xml_diff>
--- a/v2/tests/fixtures/mini/FACTURAS_20260731.xlsx
+++ b/v2/tests/fixtures/mini/FACTURAS_20260731.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>617873</v>
+        <v>617686</v>
       </c>
       <c r="I2" s="1" t="n">
         <v>46264</v>
@@ -579,7 +579,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>70809304.65000001</v>
+        <v>70787889</v>
       </c>
       <c r="I3" s="1" t="n">
         <v>46265</v>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>3863732</v>
+        <v>3862506</v>
       </c>
       <c r="I4" s="1" t="n">
         <v>46266</v>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>14862770</v>
+        <v>14858275</v>
       </c>
       <c r="I5" s="1" t="n">
         <v>46267</v>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>6064868</v>
+        <v>6063034</v>
       </c>
       <c r="I6" s="1" t="n">
         <v>46268</v>
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>586259</v>
+        <v>581174</v>
       </c>
       <c r="I9" s="1" t="n">
         <v>46271</v>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>251328</v>
+        <v>249148</v>
       </c>
       <c r="I10" s="1" t="n">
         <v>46272</v>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>690200</v>
+        <v>684213</v>
       </c>
       <c r="I11" s="1" t="n">
         <v>46273</v>
@@ -1047,7 +1047,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>4066230</v>
+        <v>4032358</v>
       </c>
       <c r="I12" s="1" t="n">
         <v>46274</v>
@@ -1099,7 +1099,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>5725055</v>
+        <v>5545922</v>
       </c>
       <c r="I13" s="1" t="n">
         <v>46275</v>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>3467780</v>
+        <v>3370649</v>
       </c>
       <c r="I20" s="1" t="n">
         <v>46282</v>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>3385938</v>
+        <v>3291099</v>
       </c>
       <c r="I21" s="1" t="n">
         <v>46283</v>
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>3025614</v>
+        <v>2940868</v>
       </c>
       <c r="I22" s="1" t="n">
         <v>46284</v>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>28620232</v>
+        <v>28287570</v>
       </c>
       <c r="I23" s="1" t="n">
         <v>46285</v>
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>2427326</v>
+        <v>2399113</v>
       </c>
       <c r="I24" s="1" t="n">
         <v>46286</v>
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>18407893</v>
+        <v>18193932</v>
       </c>
       <c r="I25" s="1" t="n">
         <v>46287</v>
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>19585460</v>
+        <v>19357812</v>
       </c>
       <c r="I26" s="1" t="n">
         <v>46288</v>
@@ -1827,7 +1827,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>15315936</v>
+        <v>15137914</v>
       </c>
       <c r="I27" s="1" t="n">
         <v>46289</v>
@@ -1879,7 +1879,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>23457834</v>
+        <v>23179678</v>
       </c>
       <c r="I28" s="1" t="n">
         <v>46290</v>
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>80841755</v>
+        <v>80083101</v>
       </c>
       <c r="I29" s="1" t="n">
         <v>46291</v>
@@ -1983,7 +1983,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>37696099</v>
+        <v>37390741</v>
       </c>
       <c r="I30" s="1" t="n">
         <v>46292</v>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>56553455</v>
+        <v>56421804</v>
       </c>
       <c r="I31" s="1" t="n">
         <v>46293</v>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>266061786</v>
+        <v>265924255</v>
       </c>
       <c r="I32" s="1" t="n">
         <v>46294</v>
@@ -2139,7 +2139,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>66515446</v>
+        <v>66481063</v>
       </c>
       <c r="I33" s="1" t="n">
         <v>46295</v>
@@ -2191,7 +2191,7 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>14366227</v>
+        <v>14358801</v>
       </c>
       <c r="I34" s="1" t="n">
         <v>46296</v>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>25634903</v>
+        <v>25621652</v>
       </c>
       <c r="I35" s="1" t="n">
         <v>46297</v>
@@ -2295,7 +2295,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>13404918</v>
+        <v>13397989</v>
       </c>
       <c r="I36" s="1" t="n">
         <v>46298</v>
@@ -2347,7 +2347,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>19551313</v>
+        <v>19541207</v>
       </c>
       <c r="I37" s="1" t="n">
         <v>46299</v>
@@ -2399,7 +2399,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>31355436</v>
+        <v>31339228</v>
       </c>
       <c r="I38" s="1" t="n">
         <v>46300</v>
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>55950222</v>
+        <v>55921300</v>
       </c>
       <c r="I39" s="1" t="n">
         <v>46301</v>
@@ -2503,7 +2503,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>29257303</v>
+        <v>29242179</v>
       </c>
       <c r="I40" s="1" t="n">
         <v>46302</v>
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>3343932</v>
+        <v>3342203</v>
       </c>
       <c r="I41" s="1" t="n">
         <v>46303</v>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>111673698</v>
+        <v>111615551</v>
       </c>
       <c r="I42" s="1" t="n">
         <v>46304</v>
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>41129295</v>
+        <v>41107880</v>
       </c>
       <c r="I43" s="1" t="n">
         <v>46305</v>
@@ -2711,7 +2711,7 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>8943672</v>
+        <v>8940835</v>
       </c>
       <c r="I44" s="1" t="n">
         <v>46306</v>
@@ -2763,7 +2763,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>286657</v>
+        <v>286566</v>
       </c>
       <c r="I45" s="1" t="n">
         <v>46307</v>
@@ -2815,7 +2815,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>10316341</v>
+        <v>10313221</v>
       </c>
       <c r="I46" s="1" t="n">
         <v>46308</v>
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>10563469</v>
+        <v>10560274</v>
       </c>
       <c r="I47" s="1" t="n">
         <v>46309</v>
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>8411584</v>
+        <v>8409040</v>
       </c>
       <c r="I48" s="1" t="n">
         <v>46310</v>
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>16669822</v>
+        <v>16664780</v>
       </c>
       <c r="I49" s="1" t="n">
         <v>46311</v>
@@ -3023,7 +3023,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>18144624</v>
+        <v>18139136</v>
       </c>
       <c r="I50" s="1" t="n">
         <v>46312</v>
@@ -3075,7 +3075,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>1891724</v>
+        <v>1866864</v>
       </c>
       <c r="I51" s="1" t="n">
         <v>46313</v>
@@ -3127,7 +3127,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>8866986</v>
+        <v>8735803</v>
       </c>
       <c r="I52" s="1" t="n">
         <v>46314</v>
@@ -3179,7 +3179,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>5665441</v>
+        <v>5590988</v>
       </c>
       <c r="I53" s="1" t="n">
         <v>46315</v>
@@ -3231,7 +3231,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>6154544</v>
+        <v>6070268</v>
       </c>
       <c r="I54" s="1" t="n">
         <v>46316</v>
@@ -3283,7 +3283,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1380043</v>
+        <v>1361907</v>
       </c>
       <c r="I55" s="1" t="n">
         <v>46317</v>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>2811991</v>
+        <v>2775037</v>
       </c>
       <c r="I56" s="1" t="n">
         <v>46318</v>
@@ -3387,7 +3387,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>272871</v>
+        <v>269285</v>
       </c>
       <c r="I57" s="1" t="n">
         <v>46319</v>
@@ -3439,7 +3439,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>549548</v>
+        <v>542326</v>
       </c>
       <c r="I58" s="1" t="n">
         <v>46320</v>
@@ -3491,7 +3491,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>149977</v>
+        <v>148006</v>
       </c>
       <c r="I59" s="1" t="n">
         <v>46321</v>
@@ -3543,7 +3543,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>22454213</v>
+        <v>22066577</v>
       </c>
       <c r="I60" s="1" t="n">
         <v>46322</v>
@@ -3595,7 +3595,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>7416161</v>
+        <v>7288133</v>
       </c>
       <c r="I61" s="1" t="n">
         <v>46323</v>
@@ -3647,7 +3647,7 @@
         </is>
       </c>
       <c r="H62" t="n">
-        <v>43500293</v>
+        <v>42737430</v>
       </c>
       <c r="I62" s="1" t="n">
         <v>46264</v>
@@ -3699,7 +3699,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>10013715</v>
+        <v>9871642</v>
       </c>
       <c r="I63" s="1" t="n">
         <v>46265</v>
@@ -3751,7 +3751,7 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>14309786</v>
+        <v>14106583</v>
       </c>
       <c r="I64" s="1" t="n">
         <v>46266</v>
@@ -3803,7 +3803,7 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>13239054</v>
+        <v>13052199</v>
       </c>
       <c r="I65" s="1" t="n">
         <v>46267</v>
@@ -3855,7 +3855,7 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>15353856</v>
+        <v>15174216</v>
       </c>
       <c r="I66" s="1" t="n">
         <v>46268</v>
@@ -3907,7 +3907,7 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>26727231</v>
+        <v>26368195</v>
       </c>
       <c r="I67" s="1" t="n">
         <v>46269</v>
@@ -3959,7 +3959,7 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>13090000</v>
+        <v>12953864</v>
       </c>
       <c r="I68" s="1" t="n">
         <v>46270</v>
@@ -4011,7 +4011,7 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>13041785</v>
+        <v>12857434</v>
       </c>
       <c r="I69" s="1" t="n">
         <v>46271</v>
@@ -4063,7 +4063,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>14931525</v>
+        <v>14766532</v>
       </c>
       <c r="I70" s="1" t="n">
         <v>46272</v>
@@ -4115,7 +4115,7 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>27571931</v>
+        <v>27182783</v>
       </c>
       <c r="I71" s="1" t="n">
         <v>46273</v>
@@ -4167,7 +4167,7 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>15721650</v>
+        <v>15499708</v>
       </c>
       <c r="I72" s="1" t="n">
         <v>46274</v>
@@ -4219,7 +4219,7 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>13998993</v>
+        <v>13835205</v>
       </c>
       <c r="I73" s="1" t="n">
         <v>46275</v>
@@ -4271,7 +4271,7 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>27666310</v>
+        <v>27342614</v>
       </c>
       <c r="I74" s="1" t="n">
         <v>46276</v>
@@ -4323,7 +4323,7 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>23501925</v>
+        <v>23170076</v>
       </c>
       <c r="I75" s="1" t="n">
         <v>46277</v>
@@ -4375,7 +4375,7 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>19352433</v>
+        <v>19079235</v>
       </c>
       <c r="I76" s="1" t="n">
         <v>46278</v>
@@ -4427,7 +4427,7 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>16653179</v>
+        <v>16403501</v>
       </c>
       <c r="I77" s="1" t="n">
         <v>46279</v>
@@ -4479,7 +4479,7 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>31281115</v>
+        <v>30812563</v>
       </c>
       <c r="I78" s="1" t="n">
         <v>46280</v>
@@ -4531,7 +4531,7 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>9513336</v>
+        <v>9371171</v>
       </c>
       <c r="I79" s="1" t="n">
         <v>46281</v>
@@ -4583,7 +4583,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>13860882</v>
+        <v>13686235</v>
       </c>
       <c r="I80" s="1" t="n">
         <v>46282</v>
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>13860882</v>
+        <v>13686235</v>
       </c>
       <c r="I81" s="1" t="n">
         <v>46283</v>
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>13860882</v>
+        <v>13686235</v>
       </c>
       <c r="I82" s="1" t="n">
         <v>46284</v>
@@ -4739,7 +4739,7 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>9856044</v>
+        <v>9718059</v>
       </c>
       <c r="I83" s="1" t="n">
         <v>46285</v>
@@ -4791,7 +4791,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>219813971</v>
+        <v>216582706</v>
       </c>
       <c r="I84" s="1" t="n">
         <v>46286</v>
@@ -4843,7 +4843,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>23800000</v>
+        <v>23511227</v>
       </c>
       <c r="I85" s="1" t="n">
         <v>46287</v>
@@ -4895,7 +4895,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>29630374</v>
+        <v>29270859</v>
       </c>
       <c r="I86" s="1" t="n">
         <v>46288</v>
@@ -4947,7 +4947,7 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>64810733</v>
+        <v>63852425</v>
       </c>
       <c r="I87" s="1" t="n">
         <v>46289</v>
@@ -4999,7 +4999,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>53187097</v>
+        <v>52395644</v>
       </c>
       <c r="I88" s="1" t="n">
         <v>46290</v>
@@ -5051,7 +5051,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>9096500</v>
+        <v>8967026</v>
       </c>
       <c r="I89" s="1" t="n">
         <v>46291</v>
@@ -5103,7 +5103,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>35525070</v>
+        <v>35000280</v>
       </c>
       <c r="I90" s="1" t="n">
         <v>46292</v>
@@ -5155,7 +5155,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>33546660</v>
+        <v>33047938</v>
       </c>
       <c r="I91" s="1" t="n">
         <v>46293</v>
@@ -5207,7 +5207,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>9450001</v>
+        <v>9319906</v>
       </c>
       <c r="I92" s="1" t="n">
         <v>46294</v>
@@ -5259,7 +5259,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>10742405</v>
+        <v>10604544</v>
       </c>
       <c r="I93" s="1" t="n">
         <v>46295</v>
@@ -5311,7 +5311,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>12564722</v>
+        <v>12379502</v>
       </c>
       <c r="I94" s="1" t="n">
         <v>46296</v>
@@ -5363,7 +5363,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>22610000</v>
+        <v>22298736</v>
       </c>
       <c r="I95" s="1" t="n">
         <v>46297</v>
@@ -5415,7 +5415,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>9003440</v>
+        <v>8870717</v>
       </c>
       <c r="I96" s="1" t="n">
         <v>46298</v>
@@ -5467,7 +5467,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>10710000</v>
+        <v>10577553</v>
       </c>
       <c r="I97" s="1" t="n">
         <v>46299</v>
@@ -5519,7 +5519,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>16699106</v>
+        <v>16452652</v>
       </c>
       <c r="I98" s="1" t="n">
         <v>46300</v>
@@ -5571,7 +5571,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>14798760</v>
+        <v>14580505</v>
       </c>
       <c r="I99" s="1" t="n">
         <v>46301</v>
@@ -5623,7 +5623,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>9172493</v>
+        <v>9071901</v>
       </c>
       <c r="I100" s="1" t="n">
         <v>46302</v>
@@ -5675,7 +5675,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>31274068</v>
+        <v>30855780</v>
       </c>
       <c r="I101" s="1" t="n">
         <v>46303</v>
@@ -5727,7 +5727,7 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>38114817</v>
+        <v>37605035</v>
       </c>
       <c r="I102" s="1" t="n">
         <v>46304</v>
@@ -5779,7 +5779,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>41991270</v>
+        <v>41429641</v>
       </c>
       <c r="I103" s="1" t="n">
         <v>46305</v>
@@ -5831,7 +5831,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>47647024</v>
+        <v>47009750</v>
       </c>
       <c r="I104" s="1" t="n">
         <v>46306</v>
@@ -5883,7 +5883,7 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>41825979</v>
+        <v>41265509</v>
       </c>
       <c r="I105" s="1" t="n">
         <v>46307</v>
@@ -5935,7 +5935,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>35618414</v>
+        <v>35142021</v>
       </c>
       <c r="I106" s="1" t="n">
         <v>46308</v>
@@ -5987,7 +5987,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>29440312</v>
+        <v>29096842</v>
       </c>
       <c r="I107" s="1" t="n">
         <v>46309</v>
@@ -6039,7 +6039,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>28532933</v>
+        <v>28152558</v>
       </c>
       <c r="I108" s="1" t="n">
         <v>46310</v>
@@ -6091,7 +6091,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>12831573</v>
+        <v>12677357</v>
       </c>
       <c r="I109" s="1" t="n">
         <v>46311</v>
@@ -6143,7 +6143,7 @@
         </is>
       </c>
       <c r="H110" t="n">
-        <v>18439638</v>
+        <v>18218022</v>
       </c>
       <c r="I110" s="1" t="n">
         <v>46312</v>
@@ -6195,7 +6195,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>19592424</v>
+        <v>19356953</v>
       </c>
       <c r="I111" s="1" t="n">
         <v>46313</v>
@@ -6247,7 +6247,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>20334402</v>
+        <v>20090014</v>
       </c>
       <c r="I112" s="1" t="n">
         <v>46314</v>
@@ -6299,7 +6299,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>24186200</v>
+        <v>23895644</v>
       </c>
       <c r="I113" s="1" t="n">
         <v>46315</v>
@@ -6351,7 +6351,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>12860395</v>
+        <v>12706658</v>
       </c>
       <c r="I114" s="1" t="n">
         <v>46316</v>
@@ -6403,7 +6403,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>27263092</v>
+        <v>26937181</v>
       </c>
       <c r="I115" s="1" t="n">
         <v>46317</v>
@@ -6455,7 +6455,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>13895573</v>
+        <v>13729461</v>
       </c>
       <c r="I116" s="1" t="n">
         <v>46318</v>
@@ -6507,7 +6507,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>21080041</v>
+        <v>20841696</v>
       </c>
       <c r="I117" s="1" t="n">
         <v>46319</v>
@@ -6559,7 +6559,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>28253170</v>
+        <v>27915351</v>
       </c>
       <c r="I118" s="1" t="n">
         <v>46320</v>
@@ -6611,7 +6611,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>10866517</v>
+        <v>10745971</v>
       </c>
       <c r="I119" s="1" t="n">
         <v>46321</v>
@@ -6663,7 +6663,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>12212880</v>
+        <v>12085215</v>
       </c>
       <c r="I120" s="1" t="n">
         <v>46322</v>
@@ -6715,7 +6715,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>18148595</v>
+        <v>17947267</v>
       </c>
       <c r="I121" s="1" t="n">
         <v>46323</v>
@@ -6767,7 +6767,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>15355402</v>
+        <v>15185059</v>
       </c>
       <c r="I122" s="1" t="n">
         <v>46264</v>
@@ -6819,7 +6819,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>40945361</v>
+        <v>40483543</v>
       </c>
       <c r="I123" s="1" t="n">
         <v>46265</v>
@@ -6871,7 +6871,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>48423036</v>
+        <v>47877115</v>
       </c>
       <c r="I124" s="1" t="n">
         <v>46266</v>
@@ -6923,7 +6923,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>55549114</v>
+        <v>54922853</v>
       </c>
       <c r="I125" s="1" t="n">
         <v>46267</v>
@@ -6975,7 +6975,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>69058770</v>
+        <v>68279018</v>
       </c>
       <c r="I126" s="1" t="n">
         <v>46268</v>
@@ -7027,7 +7027,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>121730905</v>
+        <v>120355828</v>
       </c>
       <c r="I127" s="1" t="n">
         <v>46269</v>
@@ -7079,7 +7079,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>133150557</v>
+        <v>131650394</v>
       </c>
       <c r="I128" s="1" t="n">
         <v>46270</v>
@@ -7131,7 +7131,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>80673141</v>
+        <v>79756678</v>
       </c>
       <c r="I129" s="1" t="n">
         <v>46271</v>
@@ -7183,7 +7183,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>38293328</v>
+        <v>37861515</v>
       </c>
       <c r="I130" s="1" t="n">
         <v>46272</v>
@@ -7235,7 +7235,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>5227333</v>
+        <v>5148560</v>
       </c>
       <c r="I131" s="1" t="n">
         <v>46273</v>
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>17242099</v>
+        <v>16982270</v>
       </c>
       <c r="I132" s="1" t="n">
         <v>46274</v>
@@ -7339,7 +7339,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>5100962</v>
+        <v>5024093</v>
       </c>
       <c r="I133" s="1" t="n">
         <v>46275</v>
@@ -7391,7 +7391,7 @@
         </is>
       </c>
       <c r="H134" t="n">
-        <v>5569897</v>
+        <v>5485962</v>
       </c>
       <c r="I134" s="1" t="n">
         <v>46276</v>
@@ -7443,7 +7443,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>5303636</v>
+        <v>5223713</v>
       </c>
       <c r="I135" s="1" t="n">
         <v>46277</v>
@@ -7495,7 +7495,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>8213226</v>
+        <v>8089457</v>
       </c>
       <c r="I136" s="1" t="n">
         <v>46278</v>
@@ -7547,7 +7547,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>6867627</v>
+        <v>6764136</v>
       </c>
       <c r="I137" s="1" t="n">
         <v>46279</v>
@@ -7599,7 +7599,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>12883597</v>
+        <v>12746054</v>
       </c>
       <c r="I138" s="1" t="n">
         <v>46280</v>
@@ -7651,7 +7651,7 @@
         </is>
       </c>
       <c r="H139" t="n">
-        <v>9357287</v>
+        <v>9307872</v>
       </c>
       <c r="I139" s="1" t="n">
         <v>46281</v>
@@ -7703,7 +7703,7 @@
         </is>
       </c>
       <c r="H140" t="n">
-        <v>9485476</v>
+        <v>9450064</v>
       </c>
       <c r="I140" s="1" t="n">
         <v>46282</v>
@@ -7755,7 +7755,7 @@
         </is>
       </c>
       <c r="H141" t="n">
-        <v>12052282</v>
+        <v>11988886</v>
       </c>
       <c r="I141" s="1" t="n">
         <v>46283</v>
@@ -7807,7 +7807,7 @@
         </is>
       </c>
       <c r="H142" t="n">
-        <v>19845413</v>
+        <v>19740612</v>
       </c>
       <c r="I142" s="1" t="n">
         <v>46284</v>
@@ -7859,7 +7859,7 @@
         </is>
       </c>
       <c r="H143" t="n">
-        <v>20170773</v>
+        <v>20064254</v>
       </c>
       <c r="I143" s="1" t="n">
         <v>46285</v>
@@ -7911,7 +7911,7 @@
         </is>
       </c>
       <c r="H144" t="n">
-        <v>205672782</v>
+        <v>204590119</v>
       </c>
       <c r="I144" s="1" t="n">
         <v>46286</v>
@@ -7963,7 +7963,7 @@
         </is>
       </c>
       <c r="H145" t="n">
-        <v>15703281</v>
+        <v>15620728</v>
       </c>
       <c r="I145" s="1" t="n">
         <v>46287</v>
@@ -8015,7 +8015,7 @@
         </is>
       </c>
       <c r="H146" t="n">
-        <v>21515494</v>
+        <v>21402491</v>
       </c>
       <c r="I146" s="1" t="n">
         <v>46288</v>
@@ -8067,7 +8067,7 @@
         </is>
       </c>
       <c r="H147" t="n">
-        <v>159211680</v>
+        <v>158374061</v>
       </c>
       <c r="I147" s="1" t="n">
         <v>46289</v>
@@ -8119,7 +8119,7 @@
         </is>
       </c>
       <c r="H148" t="n">
-        <v>13682825</v>
+        <v>13610459</v>
       </c>
       <c r="I148" s="1" t="n">
         <v>46290</v>
@@ -8171,7 +8171,7 @@
         </is>
       </c>
       <c r="H149" t="n">
-        <v>21279821</v>
+        <v>21167275</v>
       </c>
       <c r="I149" s="1" t="n">
         <v>46291</v>
@@ -8223,7 +8223,7 @@
         </is>
       </c>
       <c r="H150" t="n">
-        <v>24761974</v>
+        <v>24631011</v>
       </c>
       <c r="I150" s="1" t="n">
         <v>46292</v>
@@ -8275,7 +8275,7 @@
         </is>
       </c>
       <c r="H151" t="n">
-        <v>29017938</v>
+        <v>28864466</v>
       </c>
       <c r="I151" s="1" t="n">
         <v>46293</v>
@@ -8327,7 +8327,7 @@
         </is>
       </c>
       <c r="H152" t="n">
-        <v>33680800</v>
+        <v>33502667</v>
       </c>
       <c r="I152" s="1" t="n">
         <v>46294</v>
@@ -8379,7 +8379,7 @@
         </is>
       </c>
       <c r="H153" t="n">
-        <v>16282033</v>
+        <v>16209089</v>
       </c>
       <c r="I153" s="1" t="n">
         <v>46295</v>
@@ -8431,7 +8431,7 @@
         </is>
       </c>
       <c r="H154" t="n">
-        <v>16282033</v>
+        <v>16209089</v>
       </c>
       <c r="I154" s="1" t="n">
         <v>46296</v>
@@ -8483,7 +8483,7 @@
         </is>
       </c>
       <c r="H155" t="n">
-        <v>21346486</v>
+        <v>21250854</v>
       </c>
       <c r="I155" s="1" t="n">
         <v>46297</v>
@@ -8535,7 +8535,7 @@
         </is>
       </c>
       <c r="H156" t="n">
-        <v>9259520</v>
+        <v>9211078</v>
       </c>
       <c r="I156" s="1" t="n">
         <v>46298</v>
@@ -8587,7 +8587,7 @@
         </is>
       </c>
       <c r="H157" t="n">
-        <v>9757808</v>
+        <v>9721379</v>
       </c>
       <c r="I157" s="1" t="n">
         <v>46299</v>
@@ -8639,7 +8639,7 @@
         </is>
       </c>
       <c r="H158" t="n">
-        <v>10886601</v>
+        <v>10829023</v>
       </c>
       <c r="I158" s="1" t="n">
         <v>46300</v>
@@ -8691,7 +8691,7 @@
         </is>
       </c>
       <c r="H159" t="n">
-        <v>64730754</v>
+        <v>64392428</v>
       </c>
       <c r="I159" s="1" t="n">
         <v>46301</v>
@@ -8743,7 +8743,7 @@
         </is>
       </c>
       <c r="H160" t="n">
-        <v>24830078</v>
+        <v>24699886</v>
       </c>
       <c r="I160" s="1" t="n">
         <v>46302</v>
@@ -8795,7 +8795,7 @@
         </is>
       </c>
       <c r="H161" t="n">
-        <v>34492150</v>
+        <v>34311871</v>
       </c>
       <c r="I161" s="1" t="n">
         <v>46303</v>
@@ -8847,7 +8847,7 @@
         </is>
       </c>
       <c r="H162" t="n">
-        <v>15447707</v>
+        <v>15366861</v>
       </c>
       <c r="I162" s="1" t="n">
         <v>46304</v>
@@ -8899,7 +8899,7 @@
         </is>
       </c>
       <c r="H163" t="n">
-        <v>11479140</v>
+        <v>11418186</v>
       </c>
       <c r="I163" s="1" t="n">
         <v>46305</v>
@@ -8951,7 +8951,7 @@
         </is>
       </c>
       <c r="H164" t="n">
-        <v>11039526</v>
+        <v>10981707</v>
       </c>
       <c r="I164" s="1" t="n">
         <v>46306</v>
@@ -9003,7 +9003,7 @@
         </is>
       </c>
       <c r="H165" t="n">
-        <v>10759084</v>
+        <v>10702671</v>
       </c>
       <c r="I165" s="1" t="n">
         <v>46307</v>
@@ -9055,7 +9055,7 @@
         </is>
       </c>
       <c r="H166" t="n">
-        <v>34794899</v>
+        <v>34617845</v>
       </c>
       <c r="I166" s="1" t="n">
         <v>46308</v>
@@ -9107,7 +9107,7 @@
         </is>
       </c>
       <c r="H167" t="n">
-        <v>12406721</v>
+        <v>12343615</v>
       </c>
       <c r="I167" s="1" t="n">
         <v>46309</v>
@@ -9159,7 +9159,7 @@
         </is>
       </c>
       <c r="H168" t="n">
-        <v>11734054</v>
+        <v>11674369</v>
       </c>
       <c r="I168" s="1" t="n">
         <v>46310</v>
@@ -9211,7 +9211,7 @@
         </is>
       </c>
       <c r="H169" t="n">
-        <v>17967037</v>
+        <v>17883011</v>
       </c>
       <c r="I169" s="1" t="n">
         <v>46311</v>
@@ -9263,7 +9263,7 @@
         </is>
       </c>
       <c r="H170" t="n">
-        <v>16471659</v>
+        <v>16387843</v>
       </c>
       <c r="I170" s="1" t="n">
         <v>46312</v>
@@ -9315,7 +9315,7 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>14265482</v>
+        <v>14192892</v>
       </c>
       <c r="I171" s="1" t="n">
         <v>46313</v>
@@ -9367,7 +9367,7 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>9212856</v>
+        <v>9165976</v>
       </c>
       <c r="I172" s="1" t="n">
         <v>46314</v>
@@ -9419,7 +9419,7 @@
         </is>
       </c>
       <c r="H173" t="n">
-        <v>13668007</v>
+        <v>13598457</v>
       </c>
       <c r="I173" s="1" t="n">
         <v>46315</v>
@@ -9471,7 +9471,7 @@
         </is>
       </c>
       <c r="H174" t="n">
-        <v>11751687</v>
+        <v>11691889</v>
       </c>
       <c r="I174" s="1" t="n">
         <v>46316</v>
@@ -9523,7 +9523,7 @@
         </is>
       </c>
       <c r="H175" t="n">
-        <v>13528513</v>
+        <v>13459673</v>
       </c>
       <c r="I175" s="1" t="n">
         <v>46317</v>
@@ -9575,7 +9575,7 @@
         </is>
       </c>
       <c r="H176" t="n">
-        <v>11117732</v>
+        <v>11061160</v>
       </c>
       <c r="I176" s="1" t="n">
         <v>46318</v>
@@ -9627,7 +9627,7 @@
         </is>
       </c>
       <c r="H177" t="n">
-        <v>13220957</v>
+        <v>13153750</v>
       </c>
       <c r="I177" s="1" t="n">
         <v>46319</v>
@@ -9679,7 +9679,7 @@
         </is>
       </c>
       <c r="H178" t="n">
-        <v>12422857</v>
+        <v>12359643</v>
       </c>
       <c r="I178" s="1" t="n">
         <v>46320</v>
@@ -9731,7 +9731,7 @@
         </is>
       </c>
       <c r="H179" t="n">
-        <v>9092001</v>
+        <v>9045755</v>
       </c>
       <c r="I179" s="1" t="n">
         <v>46321</v>
@@ -9783,7 +9783,7 @@
         </is>
       </c>
       <c r="H180" t="n">
-        <v>9748079</v>
+        <v>9698476</v>
       </c>
       <c r="I180" s="1" t="n">
         <v>46322</v>
@@ -9835,7 +9835,7 @@
         </is>
       </c>
       <c r="H181" t="n">
-        <v>9748079</v>
+        <v>9698476</v>
       </c>
       <c r="I181" s="1" t="n">
         <v>46323</v>
@@ -9887,7 +9887,7 @@
         </is>
       </c>
       <c r="H182" t="n">
-        <v>9519396</v>
+        <v>9470976</v>
       </c>
       <c r="I182" s="1" t="n">
         <v>46264</v>
@@ -9939,7 +9939,7 @@
         </is>
       </c>
       <c r="H183" t="n">
-        <v>9139501</v>
+        <v>9100475</v>
       </c>
       <c r="I183" s="1" t="n">
         <v>46265</v>
@@ -9991,7 +9991,7 @@
         </is>
       </c>
       <c r="H184" t="n">
-        <v>30657128</v>
+        <v>30506572</v>
       </c>
       <c r="I184" s="1" t="n">
         <v>46266</v>
@@ -10043,7 +10043,7 @@
         </is>
       </c>
       <c r="H185" t="n">
-        <v>9893321</v>
+        <v>9844725</v>
       </c>
       <c r="I185" s="1" t="n">
         <v>46267</v>
@@ -10095,7 +10095,7 @@
         </is>
       </c>
       <c r="H186" t="n">
-        <v>13513728</v>
+        <v>13447349</v>
       </c>
       <c r="I186" s="1" t="n">
         <v>46268</v>
@@ -10147,7 +10147,7 @@
         </is>
       </c>
       <c r="H187" t="n">
-        <v>246667160</v>
+        <v>245929483</v>
       </c>
       <c r="I187" s="1" t="n">
         <v>46269</v>
@@ -10199,7 +10199,7 @@
         </is>
       </c>
       <c r="H188" t="n">
-        <v>93290641</v>
+        <v>93010969</v>
       </c>
       <c r="I188" s="1" t="n">
         <v>46270</v>
@@ -10251,7 +10251,7 @@
         </is>
       </c>
       <c r="H189" t="n">
-        <v>66812204</v>
+        <v>66611873</v>
       </c>
       <c r="I189" s="1" t="n">
         <v>46271</v>
@@ -10303,7 +10303,7 @@
         </is>
       </c>
       <c r="H190" t="n">
-        <v>11294694</v>
+        <v>11260764</v>
       </c>
       <c r="I190" s="1" t="n">
         <v>46272</v>
@@ -10355,7 +10355,7 @@
         </is>
       </c>
       <c r="H191" t="n">
-        <v>33778174</v>
+        <v>33676703</v>
       </c>
       <c r="I191" s="1" t="n">
         <v>46273</v>
@@ -10407,7 +10407,7 @@
         </is>
       </c>
       <c r="H192" t="n">
-        <v>84989446</v>
+        <v>84734133</v>
       </c>
       <c r="I192" s="1" t="n">
         <v>46274</v>
@@ -10459,7 +10459,7 @@
         </is>
       </c>
       <c r="H193" t="n">
-        <v>140548530</v>
+        <v>140125521</v>
       </c>
       <c r="I193" s="1" t="n">
         <v>46275</v>
@@ -10511,7 +10511,7 @@
         </is>
       </c>
       <c r="H194" t="n">
-        <v>10228927</v>
+        <v>10198141</v>
       </c>
       <c r="I194" s="1" t="n">
         <v>46276</v>
@@ -10563,7 +10563,7 @@
         </is>
       </c>
       <c r="H195" t="n">
-        <v>10940718</v>
+        <v>10907783</v>
       </c>
       <c r="I195" s="1" t="n">
         <v>46277</v>
@@ -10615,7 +10615,7 @@
         </is>
       </c>
       <c r="H196" t="n">
-        <v>141986314</v>
+        <v>141558897</v>
       </c>
       <c r="I196" s="1" t="n">
         <v>46278</v>
@@ -10667,7 +10667,7 @@
         </is>
       </c>
       <c r="H197" t="n">
-        <v>130320118</v>
+        <v>129927820</v>
       </c>
       <c r="I197" s="1" t="n">
         <v>46279</v>
@@ -10719,7 +10719,7 @@
         </is>
       </c>
       <c r="H198" t="n">
-        <v>75138270</v>
+        <v>75011231</v>
       </c>
       <c r="I198" s="1" t="n">
         <v>46280</v>
@@ -10771,7 +10771,7 @@
         </is>
       </c>
       <c r="H199" t="n">
-        <v>69030633</v>
+        <v>68913921</v>
       </c>
       <c r="I199" s="1" t="n">
         <v>46281</v>
@@ -10823,7 +10823,7 @@
         </is>
       </c>
       <c r="H200" t="n">
-        <v>69659375</v>
+        <v>69541445</v>
       </c>
       <c r="I200" s="1" t="n">
         <v>46282</v>
@@ -10875,7 +10875,7 @@
         </is>
       </c>
       <c r="H201" t="n">
-        <v>43530391</v>
+        <v>43456696</v>
       </c>
       <c r="I201" s="1" t="n">
         <v>46283</v>
@@ -10927,7 +10927,7 @@
         </is>
       </c>
       <c r="H202" t="n">
-        <v>35958452</v>
+        <v>35897610</v>
       </c>
       <c r="I202" s="1" t="n">
         <v>46284</v>
@@ -10979,7 +10979,7 @@
         </is>
       </c>
       <c r="H203" t="n">
-        <v>124321395</v>
+        <v>124298084</v>
       </c>
       <c r="I203" s="1" t="n">
         <v>46285</v>
@@ -11031,7 +11031,7 @@
         </is>
       </c>
       <c r="H204" t="n">
-        <v>80625451</v>
+        <v>80610367</v>
       </c>
       <c r="I204" s="1" t="n">
         <v>46286</v>
@@ -11083,7 +11083,7 @@
         </is>
       </c>
       <c r="H205" t="n">
-        <v>51727402</v>
+        <v>51717716</v>
       </c>
       <c r="I205" s="1" t="n">
         <v>46287</v>
@@ -11135,7 +11135,7 @@
         </is>
       </c>
       <c r="H206" t="n">
-        <v>43724037</v>
+        <v>43715817</v>
       </c>
       <c r="I206" s="1" t="n">
         <v>46288</v>
@@ -11187,7 +11187,7 @@
         </is>
       </c>
       <c r="H207" t="n">
-        <v>33217978</v>
+        <v>33211756</v>
       </c>
       <c r="I207" s="1" t="n">
         <v>46289</v>
@@ -11239,7 +11239,7 @@
         </is>
       </c>
       <c r="H208" t="n">
-        <v>33209809</v>
+        <v>33203590</v>
       </c>
       <c r="I208" s="1" t="n">
         <v>46290</v>
@@ -11291,7 +11291,7 @@
         </is>
       </c>
       <c r="H209" t="n">
-        <v>29444566</v>
+        <v>29439013</v>
       </c>
       <c r="I209" s="1" t="n">
         <v>46291</v>
@@ -11343,7 +11343,7 @@
         </is>
       </c>
       <c r="H210" t="n">
-        <v>25271720</v>
+        <v>25266954</v>
       </c>
       <c r="I210" s="1" t="n">
         <v>46292</v>
@@ -11395,7 +11395,7 @@
         </is>
       </c>
       <c r="H211" t="n">
-        <v>27907061</v>
+        <v>27901814</v>
       </c>
       <c r="I211" s="1" t="n">
         <v>46293</v>
@@ -11447,7 +11447,7 @@
         </is>
       </c>
       <c r="H212" t="n">
-        <v>27564373</v>
+        <v>27559204</v>
       </c>
       <c r="I212" s="1" t="n">
         <v>46294</v>
@@ -11499,7 +11499,7 @@
         </is>
       </c>
       <c r="H213" t="n">
-        <v>26526043</v>
+        <v>26521081</v>
       </c>
       <c r="I213" s="1" t="n">
         <v>46295</v>
@@ -11551,7 +11551,7 @@
         </is>
       </c>
       <c r="H214" t="n">
-        <v>25354955</v>
+        <v>25350188</v>
       </c>
       <c r="I214" s="1" t="n">
         <v>46296</v>
@@ -11603,7 +11603,7 @@
         </is>
       </c>
       <c r="H215" t="n">
-        <v>24487027</v>
+        <v>24482429</v>
       </c>
       <c r="I215" s="1" t="n">
         <v>46297</v>
@@ -11655,7 +11655,7 @@
         </is>
       </c>
       <c r="H216" t="n">
-        <v>24459437</v>
+        <v>24454839</v>
       </c>
       <c r="I216" s="1" t="n">
         <v>46298</v>
@@ -11707,7 +11707,7 @@
         </is>
       </c>
       <c r="H217" t="n">
-        <v>24148583</v>
+        <v>24144043</v>
       </c>
       <c r="I217" s="1" t="n">
         <v>46299</v>
@@ -11759,7 +11759,7 @@
         </is>
       </c>
       <c r="H218" t="n">
-        <v>24484713</v>
+        <v>24480134</v>
       </c>
       <c r="I218" s="1" t="n">
         <v>46300</v>
@@ -11811,7 +11811,7 @@
         </is>
       </c>
       <c r="H219" t="n">
-        <v>24016074</v>
+        <v>24011569</v>
       </c>
       <c r="I219" s="1" t="n">
         <v>46301</v>
@@ -11863,7 +11863,7 @@
         </is>
       </c>
       <c r="H220" t="n">
-        <v>23953557</v>
+        <v>23949059</v>
       </c>
       <c r="I220" s="1" t="n">
         <v>46302</v>
@@ -11915,7 +11915,7 @@
         </is>
       </c>
       <c r="H221" t="n">
-        <v>23984092</v>
+        <v>23979606</v>
       </c>
       <c r="I221" s="1" t="n">
         <v>46303</v>
@@ -11967,7 +11967,7 @@
         </is>
       </c>
       <c r="H222" t="n">
-        <v>23892211</v>
+        <v>23887737</v>
       </c>
       <c r="I222" s="1" t="n">
         <v>46304</v>
@@ -12019,7 +12019,7 @@
         </is>
       </c>
       <c r="H223" t="n">
-        <v>22487127</v>
+        <v>22482894</v>
       </c>
       <c r="I223" s="1" t="n">
         <v>46305</v>
@@ -12071,7 +12071,7 @@
         </is>
       </c>
       <c r="H224" t="n">
-        <v>22165743</v>
+        <v>22161565</v>
       </c>
       <c r="I224" s="1" t="n">
         <v>46306</v>
@@ -12123,7 +12123,7 @@
         </is>
       </c>
       <c r="H225" t="n">
-        <v>18998051</v>
+        <v>18994459</v>
       </c>
       <c r="I225" s="1" t="n">
         <v>46307</v>
@@ -12175,7 +12175,7 @@
         </is>
       </c>
       <c r="H226" t="n">
-        <v>19048942</v>
+        <v>19045378</v>
       </c>
       <c r="I226" s="1" t="n">
         <v>46308</v>
@@ -12227,7 +12227,7 @@
         </is>
       </c>
       <c r="H227" t="n">
-        <v>18941803</v>
+        <v>18938256</v>
       </c>
       <c r="I227" s="1" t="n">
         <v>46309</v>
@@ -12279,7 +12279,7 @@
         </is>
       </c>
       <c r="H228" t="n">
-        <v>18165423</v>
+        <v>18162024</v>
       </c>
       <c r="I228" s="1" t="n">
         <v>46310</v>
@@ -12331,7 +12331,7 @@
         </is>
       </c>
       <c r="H229" t="n">
-        <v>42248368</v>
+        <v>41447058</v>
       </c>
       <c r="I229" s="1" t="n">
         <v>46311</v>
@@ -12383,7 +12383,7 @@
         </is>
       </c>
       <c r="H230" t="n">
-        <v>20098483</v>
+        <v>19717282</v>
       </c>
       <c r="I230" s="1" t="n">
         <v>46312</v>
@@ -12435,7 +12435,7 @@
         </is>
       </c>
       <c r="H231" t="n">
-        <v>68110780</v>
+        <v>66818947</v>
       </c>
       <c r="I231" s="1" t="n">
         <v>46313</v>
@@ -12487,7 +12487,7 @@
         </is>
       </c>
       <c r="H232" t="n">
-        <v>1282870</v>
+        <v>1258539</v>
       </c>
       <c r="I232" s="1" t="n">
         <v>46314</v>
@@ -12539,7 +12539,7 @@
         </is>
       </c>
       <c r="H233" t="n">
-        <v>439421094</v>
+        <v>434067594</v>
       </c>
       <c r="I233" s="1" t="n">
         <v>46315</v>
@@ -12591,7 +12591,7 @@
         </is>
       </c>
       <c r="H234" t="n">
-        <v>369323051</v>
+        <v>368463303</v>
       </c>
       <c r="I234" s="1" t="n">
         <v>46316</v>
@@ -12643,7 +12643,7 @@
         </is>
       </c>
       <c r="H235" t="n">
-        <v>2323870</v>
+        <v>2288427</v>
       </c>
       <c r="I235" s="1" t="n">
         <v>46317</v>
@@ -12695,7 +12695,7 @@
         </is>
       </c>
       <c r="H236" t="n">
-        <v>8243092</v>
+        <v>8117371</v>
       </c>
       <c r="I236" s="1" t="n">
         <v>46318</v>
@@ -12747,7 +12747,7 @@
         </is>
       </c>
       <c r="H237" t="n">
-        <v>2802601</v>
+        <v>2759857</v>
       </c>
       <c r="I237" s="1" t="n">
         <v>46319</v>
@@ -12799,7 +12799,7 @@
         </is>
       </c>
       <c r="H238" t="n">
-        <v>1849714</v>
+        <v>1821503</v>
       </c>
       <c r="I238" s="1" t="n">
         <v>46320</v>
@@ -12851,7 +12851,7 @@
         </is>
       </c>
       <c r="H239" t="n">
-        <v>2459991</v>
+        <v>2422472</v>
       </c>
       <c r="I239" s="1" t="n">
         <v>46321</v>
@@ -12903,7 +12903,7 @@
         </is>
       </c>
       <c r="H240" t="n">
-        <v>994359</v>
+        <v>979193</v>
       </c>
       <c r="I240" s="1" t="n">
         <v>46322</v>
@@ -12955,7 +12955,7 @@
         </is>
       </c>
       <c r="H241" t="n">
-        <v>14926928</v>
+        <v>14699268</v>
       </c>
       <c r="I241" s="1" t="n">
         <v>46323</v>
@@ -13007,7 +13007,7 @@
         </is>
       </c>
       <c r="H242" t="n">
-        <v>6705010</v>
+        <v>6602748</v>
       </c>
       <c r="I242" s="1" t="n">
         <v>46264</v>
@@ -13059,7 +13059,7 @@
         </is>
       </c>
       <c r="H243" t="n">
-        <v>5411252</v>
+        <v>5328722</v>
       </c>
       <c r="I243" s="1" t="n">
         <v>46265</v>
@@ -13111,7 +13111,7 @@
         </is>
       </c>
       <c r="H244" t="n">
-        <v>17392924</v>
+        <v>17127653</v>
       </c>
       <c r="I244" s="1" t="n">
         <v>46266</v>
@@ -13163,7 +13163,7 @@
         </is>
       </c>
       <c r="H245" t="n">
-        <v>11047846</v>
+        <v>10879348</v>
       </c>
       <c r="I245" s="1" t="n">
         <v>46267</v>
@@ -13215,7 +13215,7 @@
         </is>
       </c>
       <c r="H246" t="n">
-        <v>9912238</v>
+        <v>9761060</v>
       </c>
       <c r="I246" s="1" t="n">
         <v>46268</v>
@@ -13267,7 +13267,7 @@
         </is>
       </c>
       <c r="H247" t="n">
-        <v>26009730</v>
+        <v>25657224</v>
       </c>
       <c r="I247" s="1" t="n">
         <v>46269</v>
@@ -13319,7 +13319,7 @@
         </is>
       </c>
       <c r="H248" t="n">
-        <v>99350093</v>
+        <v>98180681</v>
       </c>
       <c r="I248" s="1" t="n">
         <v>46270</v>
@@ -13371,7 +13371,7 @@
         </is>
       </c>
       <c r="H249" t="n">
-        <v>12416627</v>
+        <v>12274223</v>
       </c>
       <c r="I249" s="1" t="n">
         <v>46271</v>
@@ -13423,7 +13423,7 @@
         </is>
       </c>
       <c r="H250" t="n">
-        <v>11797880</v>
+        <v>11669964</v>
       </c>
       <c r="I250" s="1" t="n">
         <v>46272</v>
@@ -13475,7 +13475,7 @@
         </is>
       </c>
       <c r="H251" t="n">
-        <v>9245383</v>
+        <v>9145142</v>
       </c>
       <c r="I251" s="1" t="n">
         <v>46273</v>
@@ -13527,7 +13527,7 @@
         </is>
       </c>
       <c r="H252" t="n">
-        <v>17723321</v>
+        <v>17531160</v>
       </c>
       <c r="I252" s="1" t="n">
         <v>46274</v>
@@ -13579,7 +13579,7 @@
         </is>
       </c>
       <c r="H253" t="n">
-        <v>46372280</v>
+        <v>45869499</v>
       </c>
       <c r="I253" s="1" t="n">
         <v>46275</v>
@@ -13631,7 +13631,7 @@
         </is>
       </c>
       <c r="H254" t="n">
-        <v>504084231</v>
+        <v>498607260</v>
       </c>
       <c r="I254" s="1" t="n">
         <v>46276</v>
@@ -13683,7 +13683,7 @@
         </is>
       </c>
       <c r="H255" t="n">
-        <v>504084231</v>
+        <v>498607260</v>
       </c>
       <c r="I255" s="1" t="n">
         <v>46277</v>
@@ -13735,7 +13735,7 @@
         </is>
       </c>
       <c r="H256" t="n">
-        <v>378063174</v>
+        <v>373955445</v>
       </c>
       <c r="I256" s="1" t="n">
         <v>46278</v>
@@ -13787,7 +13787,7 @@
         </is>
       </c>
       <c r="H257" t="n">
-        <v>36373000</v>
+        <v>35977800</v>
       </c>
       <c r="I257" s="1" t="n">
         <v>46279</v>
@@ -13839,7 +13839,7 @@
         </is>
       </c>
       <c r="H258" t="n">
-        <v>7696783</v>
+        <v>7628405</v>
       </c>
       <c r="I258" s="1" t="n">
         <v>46280</v>
@@ -13891,7 +13891,7 @@
         </is>
       </c>
       <c r="H259" t="n">
-        <v>4536800</v>
+        <v>4496496</v>
       </c>
       <c r="I259" s="1" t="n">
         <v>46281</v>
@@ -13943,7 +13943,7 @@
         </is>
       </c>
       <c r="H260" t="n">
-        <v>974018</v>
+        <v>965365</v>
       </c>
       <c r="I260" s="1" t="n">
         <v>46282</v>
@@ -13995,7 +13995,7 @@
         </is>
       </c>
       <c r="H261" t="n">
-        <v>2858584</v>
+        <v>2833189</v>
       </c>
       <c r="I261" s="1" t="n">
         <v>46283</v>
@@ -14047,7 +14047,7 @@
         </is>
       </c>
       <c r="H262" t="n">
-        <v>1491354</v>
+        <v>1478105</v>
       </c>
       <c r="I262" s="1" t="n">
         <v>46284</v>
@@ -14099,7 +14099,7 @@
         </is>
       </c>
       <c r="H263" t="n">
-        <v>3076295</v>
+        <v>3048965</v>
       </c>
       <c r="I263" s="1" t="n">
         <v>46285</v>
@@ -14151,7 +14151,7 @@
         </is>
       </c>
       <c r="H264" t="n">
-        <v>5955515</v>
+        <v>5902607</v>
       </c>
       <c r="I264" s="1" t="n">
         <v>46286</v>
@@ -14203,7 +14203,7 @@
         </is>
       </c>
       <c r="H265" t="n">
-        <v>1387594</v>
+        <v>1375267</v>
       </c>
       <c r="I265" s="1" t="n">
         <v>46287</v>
@@ -14255,7 +14255,7 @@
         </is>
       </c>
       <c r="H266" t="n">
-        <v>16055608</v>
+        <v>15939799</v>
       </c>
       <c r="I266" s="1" t="n">
         <v>46288</v>
@@ -14307,7 +14307,7 @@
         </is>
       </c>
       <c r="H267" t="n">
-        <v>4249006</v>
+        <v>4220665</v>
       </c>
       <c r="I267" s="1" t="n">
         <v>46289</v>
@@ -14359,7 +14359,7 @@
         </is>
       </c>
       <c r="H268" t="n">
-        <v>24208935</v>
+        <v>24047460</v>
       </c>
       <c r="I268" s="1" t="n">
         <v>46290</v>
@@ -14411,7 +14411,7 @@
         </is>
       </c>
       <c r="H269" t="n">
-        <v>14603111</v>
+        <v>14508354</v>
       </c>
       <c r="I269" s="1" t="n">
         <v>46291</v>
@@ -14463,7 +14463,7 @@
         </is>
       </c>
       <c r="H270" t="n">
-        <v>24030170</v>
+        <v>23874243</v>
       </c>
       <c r="I270" s="1" t="n">
         <v>46292</v>
@@ -14515,7 +14515,7 @@
         </is>
       </c>
       <c r="H271" t="n">
-        <v>1612842</v>
+        <v>1604099</v>
       </c>
       <c r="I271" s="1" t="n">
         <v>46293</v>
@@ -14567,7 +14567,7 @@
         </is>
       </c>
       <c r="H272" t="n">
-        <v>3186877</v>
+        <v>3169600</v>
       </c>
       <c r="I272" s="1" t="n">
         <v>46294</v>
@@ -14619,7 +14619,7 @@
         </is>
       </c>
       <c r="H273" t="n">
-        <v>1406505</v>
+        <v>1398880</v>
       </c>
       <c r="I273" s="1" t="n">
         <v>46295</v>
@@ -14671,7 +14671,7 @@
         </is>
       </c>
       <c r="H274" t="n">
-        <v>1612842</v>
+        <v>1604099</v>
       </c>
       <c r="I274" s="1" t="n">
         <v>46296</v>
@@ -14723,7 +14723,7 @@
         </is>
       </c>
       <c r="H275" t="n">
-        <v>2132151</v>
+        <v>2120592</v>
       </c>
       <c r="I275" s="1" t="n">
         <v>46297</v>
@@ -14775,7 +14775,7 @@
         </is>
       </c>
       <c r="H276" t="n">
-        <v>1619017</v>
+        <v>1610240</v>
       </c>
       <c r="I276" s="1" t="n">
         <v>46298</v>
@@ -14827,7 +14827,7 @@
         </is>
       </c>
       <c r="H277" t="n">
-        <v>2946940</v>
+        <v>2930964</v>
       </c>
       <c r="I277" s="1" t="n">
         <v>46299</v>
@@ -14879,7 +14879,7 @@
         </is>
       </c>
       <c r="H278" t="n">
-        <v>1406780</v>
+        <v>1399154</v>
       </c>
       <c r="I278" s="1" t="n">
         <v>46300</v>
@@ -14931,7 +14931,7 @@
         </is>
       </c>
       <c r="H279" t="n">
-        <v>1925505</v>
+        <v>1915067</v>
       </c>
       <c r="I279" s="1" t="n">
         <v>46301</v>
@@ -14983,7 +14983,7 @@
         </is>
       </c>
       <c r="H280" t="n">
-        <v>2443052</v>
+        <v>2429808</v>
       </c>
       <c r="I280" s="1" t="n">
         <v>46302</v>
@@ -15035,7 +15035,7 @@
         </is>
       </c>
       <c r="H281" t="n">
-        <v>2443052</v>
+        <v>2429808</v>
       </c>
       <c r="I281" s="1" t="n">
         <v>46303</v>
@@ -15087,7 +15087,7 @@
         </is>
       </c>
       <c r="H282" t="n">
-        <v>62143131</v>
+        <v>61874307</v>
       </c>
       <c r="I282" s="1" t="n">
         <v>46304</v>
@@ -15139,7 +15139,7 @@
         </is>
       </c>
       <c r="H283" t="n">
-        <v>20886382</v>
+        <v>20797377</v>
       </c>
       <c r="I283" s="1" t="n">
         <v>46305</v>
@@ -15191,7 +15191,7 @@
         </is>
       </c>
       <c r="H284" t="n">
-        <v>1499185</v>
+        <v>1492796</v>
       </c>
       <c r="I284" s="1" t="n">
         <v>46306</v>
@@ -15243,7 +15243,7 @@
         </is>
       </c>
       <c r="H285" t="n">
-        <v>871568</v>
+        <v>867893</v>
       </c>
       <c r="I285" s="1" t="n">
         <v>46307</v>
@@ -15295,7 +15295,7 @@
         </is>
       </c>
       <c r="H286" t="n">
-        <v>2688656</v>
+        <v>2677320</v>
       </c>
       <c r="I286" s="1" t="n">
         <v>46308</v>
@@ -15347,7 +15347,7 @@
         </is>
       </c>
       <c r="H287" t="n">
-        <v>1601460</v>
+        <v>1594707</v>
       </c>
       <c r="I287" s="1" t="n">
         <v>46309</v>
@@ -15399,7 +15399,7 @@
         </is>
       </c>
       <c r="H288" t="n">
-        <v>5609504</v>
+        <v>5585852</v>
       </c>
       <c r="I288" s="1" t="n">
         <v>46310</v>
@@ -15451,7 +15451,7 @@
         </is>
       </c>
       <c r="H289" t="n">
-        <v>3413342</v>
+        <v>3398950</v>
       </c>
       <c r="I289" s="1" t="n">
         <v>46311</v>
@@ -15503,7 +15503,7 @@
         </is>
       </c>
       <c r="H290" t="n">
-        <v>871568</v>
+        <v>867893</v>
       </c>
       <c r="I290" s="1" t="n">
         <v>46312</v>
@@ -15555,7 +15555,7 @@
         </is>
       </c>
       <c r="H291" t="n">
-        <v>1092343</v>
+        <v>1087737</v>
       </c>
       <c r="I291" s="1" t="n">
         <v>46313</v>
@@ -15607,7 +15607,7 @@
         </is>
       </c>
       <c r="H292" t="n">
-        <v>435648</v>
+        <v>433811</v>
       </c>
       <c r="I292" s="1" t="n">
         <v>46314</v>
@@ -15659,7 +15659,7 @@
         </is>
       </c>
       <c r="H293" t="n">
-        <v>1423309</v>
+        <v>1417308</v>
       </c>
       <c r="I293" s="1" t="n">
         <v>46315</v>
@@ -15711,7 +15711,7 @@
         </is>
       </c>
       <c r="H294" t="n">
-        <v>871568</v>
+        <v>867893</v>
       </c>
       <c r="I294" s="1" t="n">
         <v>46316</v>
@@ -15763,7 +15763,7 @@
         </is>
       </c>
       <c r="H295" t="n">
-        <v>871568</v>
+        <v>867893</v>
       </c>
       <c r="I295" s="1" t="n">
         <v>46317</v>
@@ -15815,7 +15815,7 @@
         </is>
       </c>
       <c r="H296" t="n">
-        <v>21941183</v>
+        <v>21887641</v>
       </c>
       <c r="I296" s="1" t="n">
         <v>46318</v>
@@ -15867,7 +15867,7 @@
         </is>
       </c>
       <c r="H297" t="n">
-        <v>526183133</v>
+        <v>525636180</v>
       </c>
       <c r="I297" s="1" t="n">
         <v>46319</v>
@@ -15919,7 +15919,7 @@
         </is>
       </c>
       <c r="H298" t="n">
-        <v>331552223</v>
+        <v>331207583</v>
       </c>
       <c r="I298" s="1" t="n">
         <v>46320</v>
@@ -15971,7 +15971,7 @@
         </is>
       </c>
       <c r="H299" t="n">
-        <v>13847132</v>
+        <v>13832738</v>
       </c>
       <c r="I299" s="1" t="n">
         <v>46321</v>
@@ -16023,7 +16023,7 @@
         </is>
       </c>
       <c r="H300" t="n">
-        <v>127902946</v>
+        <v>127836831</v>
       </c>
       <c r="I300" s="1" t="n">
         <v>46322</v>
@@ -16075,7 +16075,7 @@
         </is>
       </c>
       <c r="H301" t="n">
-        <v>2904181</v>
+        <v>2902680</v>
       </c>
       <c r="I301" s="1" t="n">
         <v>46323</v>
@@ -16127,7 +16127,7 @@
         </is>
       </c>
       <c r="H302" t="n">
-        <v>2904181</v>
+        <v>2902680</v>
       </c>
       <c r="I302" s="1" t="n">
         <v>46264</v>
@@ -16179,7 +16179,7 @@
         </is>
       </c>
       <c r="H303" t="n">
-        <v>1410377424</v>
+        <v>1416390000</v>
       </c>
       <c r="I303" s="1" t="n">
         <v>46265</v>

</xml_diff>